<commit_message>
Add TTS voice selector
</commit_message>
<xml_diff>
--- a/public/data/speedvoca_data.xlsx
+++ b/public/data/speedvoca_data.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="158">
   <si>
     <t>sentence</t>
   </si>
@@ -19,276 +19,472 @@
     <t>translation</t>
   </si>
   <si>
-    <t>Chris got the call late at night.</t>
-  </si>
-  <si>
-    <t>크리스는 늦은 밤 전화를 받았다.</t>
-  </si>
-  <si>
-    <t>There was no greeting and no explanation.</t>
-  </si>
-  <si>
-    <t>인사도, 설명도 없었다.</t>
-  </si>
-  <si>
-    <t>The Boss said one thing: “Take Mimi out.”</t>
-  </si>
-  <si>
-    <t>보스는 한 마디만 했다. “미미를 제거해.”</t>
-  </si>
-  <si>
-    <t>Chris didn’t ask why.</t>
-  </si>
-  <si>
-    <t>크리스는 이유를 묻지 않았다.</t>
-  </si>
-  <si>
-    <t>He never did.</t>
-  </si>
-  <si>
-    <t>그는 원래 그런 사람이었다.</t>
-  </si>
-  <si>
-    <t>He checked the file again: name, location, and movement pattern.</t>
-  </si>
-  <si>
-    <t>그는 다시 파일을 확인했다. 이름, 위치, 이동 패턴.</t>
-  </si>
-  <si>
-    <t>Everything looked normal, maybe too normal.</t>
-  </si>
-  <si>
-    <t>모든 게 평범해 보였다. 어쩌면 너무 평범했다.</t>
-  </si>
-  <si>
-    <t>Chris grabbed his coat and left.</t>
-  </si>
-  <si>
-    <t>크리스는 코트를 집어 들고 나갔다.</t>
-  </si>
-  <si>
-    <t>Mimi felt something was off the moment she stepped outside.</t>
-  </si>
-  <si>
-    <t>미미는 밖으로 나오는 순간 이상함을 느꼈다.</t>
-  </si>
-  <si>
-    <t>The street was quiet, but it didn’t feel safe.</t>
-  </si>
-  <si>
-    <t>거리는 조용했지만 안전하게 느껴지지 않았다.</t>
-  </si>
-  <si>
-    <t>She knew someone was nearby.</t>
-  </si>
-  <si>
-    <t>누군가 근처에 있다는 걸 알았다.</t>
-  </si>
-  <si>
-    <t>She turned a corner, and footsteps followed.</t>
-  </si>
-  <si>
-    <t>그녀가 모퉁이를 돌자 발소리가 따라왔다.</t>
-  </si>
-  <si>
-    <t>They were not fast and not loud.</t>
-  </si>
-  <si>
-    <t>빠르지도, 시끄럽지도 않았다.</t>
-  </si>
-  <si>
-    <t>They were controlled.</t>
-  </si>
-  <si>
-    <t>통제된 움직임이었다.</t>
-  </si>
-  <si>
-    <t>Mimi didn’t run right away.</t>
-  </si>
-  <si>
-    <t>미미는 바로 뛰지 않았다.</t>
-  </si>
-  <si>
-    <t>Running too early gets you caught.</t>
-  </si>
-  <si>
-    <t>너무 빨리 달리면 잡힌다.</t>
-  </si>
-  <si>
-    <t>A knife flashed in the dark.</t>
-  </si>
-  <si>
-    <t>어둠 속에서 칼이 번쩍였다.</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <color theme="1"/>
-      </rPr>
-      <t xml:space="preserve">Mimi moved </t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <b/>
-        <color theme="1"/>
-      </rPr>
-      <t>just in time.</t>
-    </r>
-  </si>
-  <si>
-    <t>미미는 간신히 피했다.</t>
-  </si>
-  <si>
-    <t>The blade missed her neck by inches.</t>
-  </si>
-  <si>
-    <t>칼날은 목을 아슬아슬하게 빗나갔다.</t>
-  </si>
-  <si>
-    <t>Chris didn’t say a word and attacked again.</t>
-  </si>
-  <si>
-    <t>크리스는 말없이 다시 공격했다.</t>
-  </si>
-  <si>
-    <t>His moves were clean and direct.</t>
-  </si>
-  <si>
-    <t>그의 움직임은 깔끔하고 직선적이었다.</t>
-  </si>
-  <si>
-    <t>Mimi blocked, slipped away, and ran.</t>
-  </si>
-  <si>
-    <t>미미는 막고, 빠져나와 달렸다.</t>
-  </si>
-  <si>
-    <t>Her leg got hit.</t>
-  </si>
-  <si>
-    <t>그녀의 다리가 베였다.</t>
-  </si>
-  <si>
-    <t>It wasn’t deep, but it slowed her down.</t>
-  </si>
-  <si>
-    <t>깊지는 않았지만 움직임이 느려졌다.</t>
-  </si>
-  <si>
-    <t>She turned into a narrow road near the fields.</t>
-  </si>
-  <si>
-    <t>그녀는 들판 근처의 좁은 길로 들어섰다.</t>
-  </si>
-  <si>
-    <t>That’s when she saw him.</t>
-  </si>
-  <si>
-    <t>그때 그녀는 그를 봤다.</t>
-  </si>
-  <si>
-    <t>His name was Karil.</t>
-  </si>
-  <si>
-    <t>그의 이름은 카릴이었다.</t>
-  </si>
-  <si>
-    <t>He was walking home after work, tired and distracted.</t>
-  </si>
-  <si>
-    <t>그는 일하고 집으로 돌아가는 길이었고, 지쳐 있었다.</t>
-  </si>
-  <si>
-    <t>He saw Mimi stumble.</t>
-  </si>
-  <si>
-    <t>그는 미미가 비틀거리는 걸 봤다.</t>
-  </si>
-  <si>
-    <t>Then he saw the man behind her with a knife.</t>
-  </si>
-  <si>
-    <t>그리고 칼을 든 남자를 봤다.</t>
-  </si>
-  <si>
-    <t>Chris stopped when he noticed a civilian.</t>
-  </si>
-  <si>
-    <t>크리스는 민간인을 보자 멈췄다.</t>
-  </si>
-  <si>
-    <t>Karil didn’t think and stepped in.</t>
-  </si>
-  <si>
-    <t>카릴은 생각하지 않고 나섰다.</t>
-  </si>
-  <si>
-    <t>He dropped what he was holding and shouted, “Hey!”</t>
-  </si>
-  <si>
-    <t>그는 들고 있던 걸 떨어뜨리며 “이봐!”라고 외쳤다.</t>
-  </si>
-  <si>
-    <t>That was enough to change things.</t>
-  </si>
-  <si>
-    <t>그 한마디로 상황이 바뀌었다.</t>
-  </si>
-  <si>
-    <t>Chris backed off.</t>
-  </si>
-  <si>
-    <t>크리스는 물러섰다.</t>
-  </si>
-  <si>
-    <t>Not because he was scared, but because it wasn’t worth it.</t>
-  </si>
-  <si>
-    <t>겁이 나서가 아니라, 그럴 가치가 없었기 때문이다.</t>
-  </si>
-  <si>
-    <t>He looked at Mimi one last time and disappeared.</t>
-  </si>
-  <si>
-    <t>그는 미미를 한 번 더 보고 사라졌다.</t>
-  </si>
-  <si>
-    <t>Mimi collapsed after he left.</t>
-  </si>
-  <si>
-    <t>그가 떠난 뒤 미미는 쓰러졌다.</t>
-  </si>
-  <si>
-    <t>Karil caught her before she hit the ground.</t>
-  </si>
-  <si>
-    <t>카릴은 그녀가 바닥에 떨어지기 전에 붙잡았다.</t>
-  </si>
-  <si>
-    <t>He said, “You’re hurt. You can’t stay here.”</t>
-  </si>
-  <si>
-    <t>그는 말했다. “다쳤어요. 여기 있으면 안 돼요.”</t>
-  </si>
-  <si>
-    <t>Mimi tried to stand, but she couldn’t.</t>
-  </si>
-  <si>
-    <t>미미는 일어서려 했지만 실패했다.</t>
-  </si>
-  <si>
-    <t>Karil hesitated for a moment.</t>
-  </si>
-  <si>
-    <t>카릴은 잠시 망설였다.</t>
-  </si>
-  <si>
-    <t>Then he said, “My place is close. Come with me.”</t>
-  </si>
-  <si>
-    <t>그리고 말했다. “제 집이 가까워요. 같이 가요.”</t>
+    <t>Should I do this now?</t>
+  </si>
+  <si>
+    <t>지금 이거 해야 해?</t>
+  </si>
+  <si>
+    <t>Do you want me to start this?</t>
+  </si>
+  <si>
+    <t>이거 내가 시작할까?</t>
+  </si>
+  <si>
+    <t>Can I start this now?</t>
+  </si>
+  <si>
+    <t>지금 시작해도 돼?</t>
+  </si>
+  <si>
+    <t>Am I doing this one?</t>
+  </si>
+  <si>
+    <t>이거 내가 하는 거야?</t>
+  </si>
+  <si>
+    <t>Should this be done now or later?</t>
+  </si>
+  <si>
+    <t>이거 지금 해야 해 아니면 나중에?</t>
+  </si>
+  <si>
+    <t>Do you want this now?</t>
+  </si>
+  <si>
+    <t>이거 지금 필요해?</t>
+  </si>
+  <si>
+    <t>Is it okay if I do this now?</t>
+  </si>
+  <si>
+    <t>지금 이거 해도 될까?</t>
+  </si>
+  <si>
+    <t>Is this a new order?</t>
+  </si>
+  <si>
+    <t>이거 새 주문이야?</t>
+  </si>
+  <si>
+    <t>Is this for the same order?</t>
+  </si>
+  <si>
+    <t>같은 주문이야?</t>
+  </si>
+  <si>
+    <t>Is this a different order?</t>
+  </si>
+  <si>
+    <t>다른 주문이야?</t>
+  </si>
+  <si>
+    <t>Did this just come in?</t>
+  </si>
+  <si>
+    <t>이거 방금 들어온 주문이야?</t>
+  </si>
+  <si>
+    <t>Which ticket is this for?</t>
+  </si>
+  <si>
+    <t>이거 어느 주문 티켓이야?</t>
+  </si>
+  <si>
+    <t>Is this for table 3?</t>
+  </si>
+  <si>
+    <t>이거 테이블 3 주문이야?</t>
+  </si>
+  <si>
+    <t>Is this the next order?</t>
+  </si>
+  <si>
+    <t>이거 다음 주문이야?</t>
+  </si>
+  <si>
+    <t>What should I do first?</t>
+  </si>
+  <si>
+    <t>뭐부터 해야 해?</t>
+  </si>
+  <si>
+    <t>Which one should I start with?</t>
+  </si>
+  <si>
+    <t>어떤 것부터 시작할까?</t>
+  </si>
+  <si>
+    <t>Should I finish this first?</t>
+  </si>
+  <si>
+    <t>이거 먼저 끝낼까?</t>
+  </si>
+  <si>
+    <t>Do you want this first or that first?</t>
+  </si>
+  <si>
+    <t>이거 먼저야 아니면 저거?</t>
+  </si>
+  <si>
+    <t>What’s the priority right now?</t>
+  </si>
+  <si>
+    <t>지금 우선순위가 뭐야?</t>
+  </si>
+  <si>
+    <t>Should I start the noodles first?</t>
+  </si>
+  <si>
+    <t>면부터 시작할까?</t>
+  </si>
+  <si>
+    <t>Do you need this first?</t>
+  </si>
+  <si>
+    <t>이거 먼저 필요해?</t>
+  </si>
+  <si>
+    <t>I did it because ~</t>
+  </si>
+  <si>
+    <t>~라서 그렇게 했어</t>
+  </si>
+  <si>
+    <t>I thought that was the order.</t>
+  </si>
+  <si>
+    <t>그렇게 하라는 주문인 줄 알았어</t>
+  </si>
+  <si>
+    <t>I thought we needed it.</t>
+  </si>
+  <si>
+    <t>우리가 그게 필요한 줄 알았어</t>
+  </si>
+  <si>
+    <t>That’s what I heard.</t>
+  </si>
+  <si>
+    <t>나는 그렇게 들었어</t>
+  </si>
+  <si>
+    <t>I thought that was correct.</t>
+  </si>
+  <si>
+    <t>그게 맞는 줄 알았어</t>
+  </si>
+  <si>
+    <t>That’s what I understood.</t>
+  </si>
+  <si>
+    <t>나는 그렇게 이해했어</t>
+  </si>
+  <si>
+    <t>I heard we should do it this way.</t>
+  </si>
+  <si>
+    <t>이렇게 해야 한다고 들었어</t>
+  </si>
+  <si>
+    <t>Is something wrong?</t>
+  </si>
+  <si>
+    <t>문제 있어?</t>
+  </si>
+  <si>
+    <t>Something seems off.</t>
+  </si>
+  <si>
+    <t>뭔가 이상해</t>
+  </si>
+  <si>
+    <t>This doesn’t look right.</t>
+  </si>
+  <si>
+    <t>이거 뭔가 이상한데</t>
+  </si>
+  <si>
+    <t>This isn’t working.</t>
+  </si>
+  <si>
+    <t>이거 작동 안 해</t>
+  </si>
+  <si>
+    <t>I think there’s a problem.</t>
+  </si>
+  <si>
+    <t>문제 있는 것 같아</t>
+  </si>
+  <si>
+    <t>This looks different.</t>
+  </si>
+  <si>
+    <t>이거 뭔가 다른데</t>
+  </si>
+  <si>
+    <t>Is this correct?</t>
+  </si>
+  <si>
+    <t>이거 맞아?</t>
+  </si>
+  <si>
+    <t>I prepared this just in case.</t>
+  </si>
+  <si>
+    <t>혹시 몰라서 준비해 놨어</t>
+  </si>
+  <si>
+    <t>I got this ready just in case.</t>
+  </si>
+  <si>
+    <t>필요할까봐 준비해 놨어</t>
+  </si>
+  <si>
+    <t>I made an extra one just in case.</t>
+  </si>
+  <si>
+    <t>혹시 몰라서 하나 더 만들었어</t>
+  </si>
+  <si>
+    <t>I thought we might need this.</t>
+  </si>
+  <si>
+    <t>필요할 것 같아서 준비했어</t>
+  </si>
+  <si>
+    <t>I set this aside just in case.</t>
+  </si>
+  <si>
+    <t>혹시 몰라서 따로 빼놨어</t>
+  </si>
+  <si>
+    <t>I kept this ready.</t>
+  </si>
+  <si>
+    <t>이거 준비해 놨어</t>
+  </si>
+  <si>
+    <t>We’re out of ~</t>
+  </si>
+  <si>
+    <t>~ 다 떨어졌어</t>
+  </si>
+  <si>
+    <t>There’s no more ~</t>
+  </si>
+  <si>
+    <t>~ 더 없어</t>
+  </si>
+  <si>
+    <t>We don’t have any left.</t>
+  </si>
+  <si>
+    <t>남은 게 없어</t>
+  </si>
+  <si>
+    <t>We’re running low on ~</t>
+  </si>
+  <si>
+    <t>~ 거의 다 떨어졌어</t>
+  </si>
+  <si>
+    <t>Do we have more ~ ?</t>
+  </si>
+  <si>
+    <t>~ 더 있어?</t>
+  </si>
+  <si>
+    <t>Where is the ~ ?</t>
+  </si>
+  <si>
+    <t>~ 어디 있어?</t>
+  </si>
+  <si>
+    <t>Is there more ~ ?</t>
+  </si>
+  <si>
+    <t>What’s going on?</t>
+  </si>
+  <si>
+    <t>무슨 상황이야?</t>
+  </si>
+  <si>
+    <t>What happened?</t>
+  </si>
+  <si>
+    <t>무슨 일 있었어?</t>
+  </si>
+  <si>
+    <t>Why did that happen?</t>
+  </si>
+  <si>
+    <t>왜 그런 일이 생긴 거야?</t>
+  </si>
+  <si>
+    <t>Why did you do that?</t>
+  </si>
+  <si>
+    <t>왜 그렇게 했어?</t>
+  </si>
+  <si>
+    <t>What should we do in this case?</t>
+  </si>
+  <si>
+    <t>이런 경우에는 어떻게 해야 해?</t>
+  </si>
+  <si>
+    <t>What do we do if that happens?</t>
+  </si>
+  <si>
+    <t>그런 일이 생기면 어떻게 해?</t>
+  </si>
+  <si>
+    <t>How many people?</t>
+  </si>
+  <si>
+    <t>몇 분이세요?</t>
+  </si>
+  <si>
+    <t>How many in your party?</t>
+  </si>
+  <si>
+    <t>Table for two?</t>
+  </si>
+  <si>
+    <t>두 분이세요?</t>
+  </si>
+  <si>
+    <t>Just one?</t>
+  </si>
+  <si>
+    <t>한 분이세요?</t>
+  </si>
+  <si>
+    <t>Right this way.</t>
+  </si>
+  <si>
+    <t>이쪽으로 오세요.</t>
+  </si>
+  <si>
+    <t>Please follow me.</t>
+  </si>
+  <si>
+    <t>이쪽으로 따라오세요.</t>
+  </si>
+  <si>
+    <t>You can sit here.</t>
+  </si>
+  <si>
+    <t>여기 앉으시면 됩니다.</t>
+  </si>
+  <si>
+    <t>This table is fine?</t>
+  </si>
+  <si>
+    <t>이 자리 괜찮으세요?</t>
+  </si>
+  <si>
+    <t>Here’s the menu.</t>
+  </si>
+  <si>
+    <t>메뉴입니다.</t>
+  </si>
+  <si>
+    <t>Are you ready to order?</t>
+  </si>
+  <si>
+    <t>주문하시겠어요?</t>
+  </si>
+  <si>
+    <t>Can I take your order?</t>
+  </si>
+  <si>
+    <t>주문 도와드릴까요?</t>
+  </si>
+  <si>
+    <t>What would you like?</t>
+  </si>
+  <si>
+    <t>무엇을 드시겠어요?</t>
+  </si>
+  <si>
+    <t>Anything to drink?</t>
+  </si>
+  <si>
+    <t>음료 필요하세요?</t>
+  </si>
+  <si>
+    <t>So that’s one tonkotsu ramen.</t>
+  </si>
+  <si>
+    <t>돈코츠 라멘 하나 맞으시죠.</t>
+  </si>
+  <si>
+    <t>Anything else?</t>
+  </si>
+  <si>
+    <t>더 필요하세요?</t>
+  </si>
+  <si>
+    <t>No green onion, right?</t>
+  </si>
+  <si>
+    <t>파는 빼는 거 맞으시죠?</t>
+  </si>
+  <si>
+    <t>Extra noodles?</t>
+  </si>
+  <si>
+    <t>면 추가하시겠어요?</t>
+  </si>
+  <si>
+    <t>Here you go.</t>
+  </si>
+  <si>
+    <t>여기 있습니다.</t>
+  </si>
+  <si>
+    <t>Enjoy your meal.</t>
+  </si>
+  <si>
+    <t>맛있게 드세요.</t>
+  </si>
+  <si>
+    <t>Be careful, it’s hot.</t>
+  </si>
+  <si>
+    <t>뜨거우니까 조심하세요.</t>
+  </si>
+  <si>
+    <t>Everything okay?</t>
+  </si>
+  <si>
+    <t>괜찮으세요?</t>
+  </si>
+  <si>
+    <t>Do you need anything?</t>
+  </si>
+  <si>
+    <t>필요한 거 있으세요?</t>
+  </si>
+  <si>
+    <t>Thank you.</t>
+  </si>
+  <si>
+    <t>감사합니다.</t>
+  </si>
+  <si>
+    <t>Have a nice day.</t>
+  </si>
+  <si>
+    <t>좋은 하루 보내세요.</t>
+  </si>
+  <si>
+    <t>See you next time.</t>
+  </si>
+  <si>
+    <t>다음에 또 오세요.</t>
   </si>
 </sst>
 </file>
@@ -311,7 +507,6 @@
     <font>
       <color theme="1"/>
       <name val="Arial"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -328,7 +523,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -336,7 +531,10 @@
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment vertical="bottom"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -911,6 +1109,294 @@
         <v>87</v>
       </c>
     </row>
+    <row r="45">
+      <c r="A45" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="B45" s="3" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="B46" s="3" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="B47" s="3" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="B48" s="3" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="B49" s="3" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="B50" s="3" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="B51" s="3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="B52" s="3" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="B53" s="3" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="B54" s="3" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="B55" s="3" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="B56" s="3" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="B57" s="3" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="B58" s="3" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="B59" s="3" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="B60" s="3" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="B61" s="3" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="B62" s="3" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="B63" s="3" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="B64" s="3" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="B65" s="3" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="B66" s="3" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="B67" s="3" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="B68" s="3" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="B69" s="3" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="B70" s="3" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="B71" s="3" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="B72" s="3" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="B73" s="3" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="B74" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="B75" s="3" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="B76" s="3" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="B77" s="3" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="B78" s="3" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="B79" s="3" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="B80" s="3" t="s">
+        <v>157</v>
+      </c>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>